<commit_message>
setup driver factory for parallel execution
</commit_message>
<xml_diff>
--- a/src/main/resources/testData/TestData.xlsx
+++ b/src/main/resources/testData/TestData.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="112">
   <si>
     <t xml:space="preserve">Function</t>
   </si>
@@ -46,10 +46,16 @@
     <t xml:space="preserve">Password123!</t>
   </si>
   <si>
+    <t xml:space="preserve">john</t>
+  </si>
+  <si>
     <t xml:space="preserve">rakesh13595@gmail.com</t>
   </si>
   <si>
     <t xml:space="preserve">Test@001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rakesh</t>
   </si>
   <si>
     <t xml:space="preserve">testCaseSensitivityEmail</t>
@@ -412,6 +418,7 @@
       <color rgb="FF000000"/>
       <name val="Monospace"/>
       <family val="0"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -769,24 +776,30 @@
       <c r="C2" s="3" t="s">
         <v>6</v>
       </c>
+      <c r="D2" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>6</v>
@@ -794,7 +807,7 @@
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>5</v>
@@ -805,10 +818,10 @@
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>6</v>
@@ -816,7 +829,7 @@
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>5</v>
@@ -827,189 +840,189 @@
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B18" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>36</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -1048,19 +1061,19 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>3</v>
@@ -1068,16 +1081,16 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>6</v>
@@ -1088,96 +1101,96 @@
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>6</v>
@@ -1188,13 +1201,13 @@
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>5</v>
@@ -1208,24 +1221,24 @@
     </row>
     <row r="9" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>6</v>
@@ -1234,18 +1247,18 @@
         <v>6</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>5</v>
@@ -1257,18 +1270,18 @@
         <v>6</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>5</v>
@@ -1277,44 +1290,44 @@
         <v>6</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="E13" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>31</v>
-      </c>
       <c r="G13" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>5</v>
@@ -1326,18 +1339,18 @@
         <v>6</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>5</v>
@@ -1349,18 +1362,18 @@
         <v>6</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>5</v>
@@ -1372,64 +1385,64 @@
         <v>6</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>5</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>5</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>5</v>
@@ -1441,18 +1454,18 @@
         <v>6</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>5</v>
@@ -1464,7 +1477,7 @@
         <v>6</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1504,20 +1517,20 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1528,23 +1541,23 @@
         <v>1</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1580,7 +1593,7 @@
         <v>2</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>3</v>
@@ -1588,7 +1601,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>6</v>
@@ -1599,36 +1612,36 @@
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>6</v>
@@ -1637,49 +1650,49 @@
         <v>6</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated TestData and changes in testcase
Added registration Test Data and changes in test cases
</commit_message>
<xml_diff>
--- a/src/main/resources/testData/TestData.xlsx
+++ b/src/main/resources/testData/TestData.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="130">
   <si>
     <t>Function</t>
   </si>
@@ -411,12 +411,44 @@
   <si>
     <t xml:space="preserve">  </t>
   </si>
+  <si>
+    <t>testPasswordErrorChecks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+password
+PASSWORD
+Password
+Password123</t>
+  </si>
+  <si>
+    <t>Password is required.
+Must include at least one uppercase letter (A-Z).
+Must include at least one lowercase letter (a-z).
+Must include at least one number (0-9).
+Must include at least one special character (@$!%*?&amp;).</t>
+  </si>
+  <si>
+    <t>Doe</t>
+  </si>
+  <si>
+    <t>john.doe@exampl
+john.doe
+@example.com
+john.doe@.com
+john..doe@example.com</t>
+  </si>
+  <si>
+    <t>Avinash.Noop_Doddu@example.com
+Avinash.Noop-Doddu@example.com
+Avinash.Noop+Doddu@example.com</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="5">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -449,6 +481,26 @@
       <name val="Arial"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -477,7 +529,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
@@ -491,6 +543,14 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1165,7 +1225,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="34.42578125" style="1" customWidth="1"/>
@@ -1186,10 +1246,10 @@
       <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="11" t="s">
         <v>94</v>
       </c>
       <c r="G1" s="2" t="s">
@@ -1572,9 +1632,79 @@
         <v>86</v>
       </c>
     </row>
+    <row r="19" spans="1:7" ht="63.75">
+      <c r="A19" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="63.75">
+      <c r="A20" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G20" s="9" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="76.5">
+      <c r="A21" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>49</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D19" r:id="rId1"/>
+    <hyperlink ref="D21" r:id="rId2" display="Avinash.Noop_Doddu@example.com"/>
+  </hyperlinks>
   <pageMargins left="0.74791666666666701" right="0.74791666666666701" top="0.98402777777777795" bottom="0.98402777777777795" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId3"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Updates on all Test's
1) added more test case to logout test.
2) error correction on create account test
3) moved some test case from login to forgot test.
</commit_message>
<xml_diff>
--- a/src/main/resources/testData/TestData.xlsx
+++ b/src/main/resources/testData/TestData.xlsx
@@ -10,7 +10,7 @@
     <sheet name="LoginTest" sheetId="1" r:id="rId1"/>
     <sheet name="CreateAccountTest" sheetId="2" r:id="rId2"/>
     <sheet name="ForgotPasswordTest" sheetId="3" r:id="rId3"/>
-    <sheet name="ResetPassword" sheetId="4" r:id="rId4"/>
+    <sheet name="LogoutTest" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="132">
   <si>
     <t>Function</t>
   </si>
@@ -232,16 +232,6 @@
     <t>doe</t>
   </si>
   <si>
-    <t>testEmptyFirstName</t>
-  </si>
-  <si>
-    <t>Last name is required.
-Email is required.
-Password is required.
-Please confirm your password.
-You must agree to the Terms and Conditions.</t>
-  </si>
-  <si>
     <t>testInvalidEmailFormat</t>
   </si>
   <si>
@@ -304,9 +294,6 @@
     <t>testLoginPageLink</t>
   </si>
   <si>
-    <t>Expected Error Messages</t>
-  </si>
-  <si>
     <t>testEmptyEmailField</t>
   </si>
   <si>
@@ -326,12 +313,6 @@
   </si>
   <si>
     <t>testEmptyPasswordField</t>
-  </si>
-  <si>
-    <t>Password is required.</t>
-  </si>
-  <si>
-    <t>Type should be text - Password123!</t>
   </si>
   <si>
     <t>testPasswordTooShort</t>
@@ -361,9 +342,6 @@
 email</t>
   </si>
   <si>
-    <t>verifyResetPasswordNotAccessibleAfterLogin</t>
-  </si>
-  <si>
     <t>verifySignUpNotAccessibleAfterLogin</t>
   </si>
   <si>
@@ -371,9 +349,6 @@
   </si>
   <si>
     <t>verifyDashoardPageNotAccessibleBeforeLogin</t>
-  </si>
-  <si>
-    <t>Sign in</t>
   </si>
   <si>
     <t>verifyResetPasswordTokenNotAccessibleAfterLogin</t>
@@ -443,12 +418,48 @@
 Avinash.Noop-Doddu@example.com
 Avinash.Noop+Doddu@example.com</t>
   </si>
+  <si>
+    <t>testValidEmailFormat</t>
+  </si>
+  <si>
+    <t>Avinash.Noop+Doddu@example.com
+john.doe@example.com
+punith7760kumar@gmail.com</t>
+  </si>
+  <si>
+    <t>Password is required.
+Please confirm your password.</t>
+  </si>
+  <si>
+    <t>testPasswordReset</t>
+  </si>
+  <si>
+    <t>testLogoutPage</t>
+  </si>
+  <si>
+    <t>john
+Sign in to your account</t>
+  </si>
+  <si>
+    <t>verifyResetPasswordPageNotAccessableAfterLogin</t>
+  </si>
+  <si>
+    <t>First name is required.
+Last name is required.
+Email is required.
+Password is required.
+Please confirm your password.
+You must agree to the Terms and Conditions.</t>
+  </si>
+  <si>
+    <t>testEmptyAllFields</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="8">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -471,19 +482,6 @@
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Monospace"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="10"/>
-      <color theme="10"/>
-      <name val="Arial"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -499,7 +497,7 @@
       <sz val="10"/>
       <color theme="10"/>
       <name val="Arial"/>
-      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -527,9 +525,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
@@ -538,17 +536,11 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -810,8 +802,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Z30"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="12.75"/>
+  <dimension ref="A1:Z26"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29.140625" style="1" customWidth="1"/>
     <col min="2" max="3" width="44.140625" style="1" customWidth="1"/>
@@ -819,7 +811,7 @@
     <col min="5" max="26" width="34" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15">
+    <row r="1" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -833,7 +825,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="14.25">
+    <row r="2" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
@@ -843,11 +835,11 @@
       <c r="C2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="14.25">
+    <row r="3" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -857,11 +849,11 @@
       <c r="C3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="14.25">
+    <row r="4" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>11</v>
       </c>
@@ -875,7 +867,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="25.5">
+    <row r="5" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>13</v>
       </c>
@@ -885,11 +877,11 @@
       <c r="C5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="6" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="14.25">
+      <c r="D5" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>14</v>
       </c>
@@ -899,65 +891,75 @@
       <c r="C6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="25.5">
+    <row r="7" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="6" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="14.25">
+      <c r="D7" s="3" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="1" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="14.25">
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="14.25">
+        <v>102</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="25.5">
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="25.5">
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="6" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="14.25">
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>21</v>
       </c>
@@ -971,7 +973,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="14.25">
+    <row r="14" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>25</v>
       </c>
@@ -982,18 +984,20 @@
         <v>27</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="28.5">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="14.25">
+    <row r="16" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
         <v>30</v>
       </c>
@@ -1007,7 +1011,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="14.25">
+    <row r="17" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
         <v>32</v>
       </c>
@@ -1021,7 +1025,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="14.25">
+    <row r="18" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
         <v>35</v>
       </c>
@@ -1035,7 +1039,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="14.25">
+    <row r="19" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
         <v>37</v>
       </c>
@@ -1049,7 +1053,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="14.25">
+    <row r="20" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>38</v>
       </c>
@@ -1063,7 +1067,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="14.25">
+    <row r="21" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
         <v>39</v>
       </c>
@@ -1077,7 +1081,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="14.25">
+    <row r="22" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
         <v>40</v>
       </c>
@@ -1091,39 +1095,39 @@
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="14.25">
-      <c r="A23" s="5" t="s">
+    <row r="23" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" s="3" t="s">
         <v>9</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="14.25">
-      <c r="A24" s="5" t="s">
+    <row r="24" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A24" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="C24" s="3" t="s">
         <v>46</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="14.25">
+    <row r="25" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="B25" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="B25" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C25" s="3" t="s">
@@ -1133,73 +1137,17 @@
         <v>7</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="14.25">
+    <row r="26" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="B26" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="B26" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="14.25">
-      <c r="A27" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="14.25">
-      <c r="A28" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="B28" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="14.25">
-      <c r="A29" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="14.25">
-      <c r="A30" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="B30" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D30" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1213,10 +1161,6 @@
     <hyperlink ref="B7" r:id="rId6"/>
     <hyperlink ref="B25" r:id="rId7"/>
     <hyperlink ref="B26" r:id="rId8"/>
-    <hyperlink ref="B27" r:id="rId9"/>
-    <hyperlink ref="B28" r:id="rId10"/>
-    <hyperlink ref="B29" r:id="rId11"/>
-    <hyperlink ref="B30" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.74791666666666701" right="0.74791666666666701" top="0.98402777777777795" bottom="0.98402777777777795" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1226,14 +1170,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="12.75"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.42578125" style="1" customWidth="1"/>
     <col min="2" max="6" width="22" style="1" customWidth="1"/>
     <col min="7" max="7" width="49.5703125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15">
+    <row r="1" spans="1:7" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1241,22 +1185,22 @@
         <v>47</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="11" t="s">
-        <v>94</v>
+      <c r="F1" s="6" t="s">
+        <v>91</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="14.25">
+    <row r="2" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
         <v>48</v>
       </c>
@@ -1279,7 +1223,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="14.25">
+    <row r="3" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
         <v>52</v>
       </c>
@@ -1302,7 +1246,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="14.25">
+    <row r="4" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>57</v>
       </c>
@@ -1322,10 +1266,10 @@
         <v>58</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="14.25">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>59</v>
       </c>
@@ -1345,10 +1289,10 @@
         <v>58</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="14.25">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
         <v>60</v>
       </c>
@@ -1371,7 +1315,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="14.25">
+    <row r="7" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>64</v>
       </c>
@@ -1394,7 +1338,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="28.5">
+    <row r="8" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
         <v>66</v>
       </c>
@@ -1413,21 +1357,26 @@
       <c r="F8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G8" s="4" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="71.25">
+      <c r="G8" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="85.5" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="4" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
         <v>69</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="14.25">
-      <c r="A10" s="3" t="s">
-        <v>71</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>67</v>
@@ -1436,7 +1385,7 @@
         <v>68</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>6</v>
@@ -1448,9 +1397,9 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="14.25">
+    <row r="11" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>67</v>
@@ -1468,12 +1417,12 @@
         <v>6</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="14.25">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>67</v>
@@ -1491,35 +1440,35 @@
         <v>31</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="85.5">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="B13" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C13" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="D13" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="E13" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="F13" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="85.5">
+      <c r="C13" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>36</v>
@@ -1536,36 +1485,36 @@
       <c r="F14" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="G14" s="4" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="57">
+      <c r="G14" s="3" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C15" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="D15" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G15" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="C15" s="3" t="s">
+    </row>
+    <row r="16" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
         <v>79</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="14.25">
-      <c r="A16" s="3" t="s">
-        <v>81</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>67</v>
@@ -1577,47 +1526,47 @@
         <v>5</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G16" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" ht="28.5">
-      <c r="A17" s="3" t="s">
+      <c r="B17" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B17" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="G17" s="4" t="s">
+      <c r="B18" s="3" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" ht="28.5">
-      <c r="A18" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>88</v>
-      </c>
       <c r="C18" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>5</v>
@@ -1628,42 +1577,43 @@
       <c r="F18" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G18" s="4" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="63.75">
+      <c r="G18" s="3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="B19" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D19" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E19" s="10" t="s">
-        <v>125</v>
-      </c>
-      <c r="G19" s="10" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="63.75">
+      <c r="E19" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>67</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>128</v>
+        <v>120</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>121</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>6</v>
@@ -1671,30 +1621,30 @@
       <c r="F20" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="G20" s="9" t="s">
+      <c r="G20" s="3" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="76.5">
-      <c r="A21" s="9" t="s">
+    <row r="21" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A21" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D21" s="12" t="s">
-        <v>129</v>
-      </c>
-      <c r="E21" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="F21" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="G21" s="9" t="s">
+      <c r="D21" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G21" s="3" t="s">
         <v>49</v>
       </c>
     </row>
@@ -1710,71 +1660,239 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D7"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="12.75"/>
+  <dimension ref="A1:E16"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="29.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="28.85546875" style="1" customWidth="1"/>
-    <col min="3" max="4" width="20.140625" style="1" customWidth="1"/>
+    <col min="1" max="2" width="29.42578125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="28.85546875" style="1" customWidth="1"/>
+    <col min="4" max="5" width="20.140625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="14.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="E1" s="6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="14.25">
+    <row r="2" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="14.25">
-      <c r="A3" s="3" t="s">
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="14.25">
-      <c r="A4" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="14.25">
+    <row r="5" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="14.25">
+        <v>70</v>
+      </c>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="57" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="B7" s="3"/>
+      <c r="C7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="14.25">
-      <c r="A7" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>72</v>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="57" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="4" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A14" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A15" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" s="3"/>
+      <c r="C15" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B5" r:id="rId1"/>
+    <hyperlink ref="B16" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.74791666666666701" right="0.74791666666666701" top="0.98402777777777795" bottom="0.98402777777777795" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -1782,127 +1900,107 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="12.75"/>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="26.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.42578125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="34.28515625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="14.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="14.25">
-      <c r="A2" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="14.25">
-      <c r="A3" s="3" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="14.25">
+    <row r="2" spans="1:4" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>129</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="14.25">
+        <v>104</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>60</v>
+        <v>105</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>63</v>
+        <v>5</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="14.25">
+        <v>6</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>98</v>
+        <v>106</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>6</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="14.25">
-      <c r="A7" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="14.25">
-      <c r="A8" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="14.25">
-      <c r="A9" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="14.25">
-      <c r="A10" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>83</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.74791666666666701" right="0.74791666666666701" top="0.98402777777777795" bottom="0.98402777777777795" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1"/>
+    <hyperlink ref="B3" r:id="rId2"/>
+    <hyperlink ref="B4" r:id="rId3"/>
+    <hyperlink ref="B5" r:id="rId4"/>
+    <hyperlink ref="B6" r:id="rId5"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Test Case on Dashboard
Added dashboard test and page.
</commit_message>
<xml_diff>
--- a/src/main/resources/testData/TestData.xlsx
+++ b/src/main/resources/testData/TestData.xlsx
@@ -4,13 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2445" windowWidth="15465" windowHeight="3030" tabRatio="500" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="2445" windowWidth="15465" windowHeight="3030" tabRatio="500" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="LoginTest" sheetId="1" r:id="rId1"/>
     <sheet name="CreateAccountTest" sheetId="2" r:id="rId2"/>
     <sheet name="ForgotPasswordTest" sheetId="3" r:id="rId3"/>
     <sheet name="LogoutTest" sheetId="4" r:id="rId4"/>
+    <sheet name="DashboardTest" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="138">
   <si>
     <t>Function</t>
   </si>
@@ -453,6 +454,27 @@
   </si>
   <si>
     <t>testEmptyAllFields</t>
+  </si>
+  <si>
+    <t>testDashboardPage</t>
+  </si>
+  <si>
+    <t>My Tasks
+john
+Sign in to your account</t>
+  </si>
+  <si>
+    <t>testTaskHomeProfilePage</t>
+  </si>
+  <si>
+    <t>testVerfiySideButton</t>
+  </si>
+  <si>
+    <t>testVerfiyAddTaskButton</t>
+  </si>
+  <si>
+    <t>john
+My Tasks</t>
   </si>
 </sst>
 </file>
@@ -527,7 +549,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
@@ -541,6 +563,13 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -939,13 +968,13 @@
         <v>101</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>19</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
-      <c r="D11" s="3" t="s">
+      <c r="D11" s="4" t="s">
         <v>103</v>
       </c>
     </row>
@@ -1443,7 +1472,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" ht="85.5" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>110</v>
       </c>
@@ -1462,7 +1491,7 @@
       <c r="F13" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="G13" s="4" t="s">
         <v>112</v>
       </c>
     </row>
@@ -1625,7 +1654,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" ht="99.75" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
         <v>64</v>
       </c>
@@ -1635,7 +1664,7 @@
       <c r="C21" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="4" t="s">
         <v>122</v>
       </c>
       <c r="E21" s="3" t="s">
@@ -2003,4 +2032,98 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A3" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>137</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1"/>
+    <hyperlink ref="B3" r:id="rId2"/>
+    <hyperlink ref="B4" r:id="rId3"/>
+    <hyperlink ref="D4" r:id="rId4"/>
+    <hyperlink ref="B5" r:id="rId5"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId6"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Changes to locator and dashboard page- 1/2 no need to merge need to check all the testcase working.
Made common file for locator, and moved the locator to their respective pages. added dashboard page.
no need to merge need to check all the testcase working.
</commit_message>
<xml_diff>
--- a/src/main/resources/testData/TestData.xlsx
+++ b/src/main/resources/testData/TestData.xlsx
@@ -241,9 +241,6 @@
     <t>testEmailAlreadyRegistered</t>
   </si>
   <si>
-    <t>Email already registered</t>
-  </si>
-  <si>
     <t>testPasswordMismatch</t>
   </si>
   <si>
@@ -453,6 +450,9 @@
   </si>
   <si>
     <t>testEmptyAllFields</t>
+  </si>
+  <si>
+    <t>Email already registered.</t>
   </si>
 </sst>
 </file>
@@ -878,7 +878,7 @@
         <v>6</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
@@ -906,7 +906,7 @@
         <v>6</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
@@ -916,17 +916,17 @@
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
@@ -936,7 +936,7 @@
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
@@ -946,7 +946,7 @@
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
@@ -956,7 +956,7 @@
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
@@ -984,7 +984,7 @@
         <v>27</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
@@ -1125,7 +1125,7 @@
     </row>
     <row r="25" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>5</v>
@@ -1139,7 +1139,7 @@
     </row>
     <row r="26" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>5</v>
@@ -1185,7 +1185,7 @@
         <v>47</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>1</v>
@@ -1194,7 +1194,7 @@
         <v>2</v>
       </c>
       <c r="F1" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>3</v>
@@ -1266,7 +1266,7 @@
         <v>58</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
@@ -1289,7 +1289,7 @@
         <v>58</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
@@ -1358,12 +1358,12 @@
         <v>6</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="85.5" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -1371,7 +1371,7 @@
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
       <c r="G9" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
@@ -1417,12 +1417,12 @@
         <v>6</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>72</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>67</v>
@@ -1440,35 +1440,35 @@
         <v>31</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>33</v>
       </c>
       <c r="C13" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="G13" s="3" t="s">
         <v>111</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>36</v>
@@ -1486,35 +1486,35 @@
         <v>36</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="C15" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="D15" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G15" s="3" t="s">
         <v>77</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>67</v>
@@ -1526,47 +1526,47 @@
         <v>5</v>
       </c>
       <c r="E16" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="G16" s="3" t="s">
         <v>80</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G17" s="3" t="s">
         <v>83</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B18" s="3" t="s">
-        <v>86</v>
-      </c>
       <c r="C18" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D18" s="3" t="s">
         <v>5</v>
@@ -1578,12 +1578,12 @@
         <v>6</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>49</v>
@@ -1595,11 +1595,11 @@
         <v>51</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F19" s="3"/>
       <c r="G19" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
@@ -1610,10 +1610,10 @@
         <v>67</v>
       </c>
       <c r="C20" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>120</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>121</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>6</v>
@@ -1636,7 +1636,7 @@
         <v>61</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>6</v>
@@ -1679,7 +1679,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E1" s="6" t="s">
         <v>3</v>
@@ -1687,35 +1687,35 @@
     </row>
     <row r="2" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A3" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
       <c r="E4" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
@@ -1733,11 +1733,11 @@
     </row>
     <row r="6" spans="1:5" ht="57" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>123</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>124</v>
-      </c>
       <c r="C6" s="3" t="s">
         <v>6</v>
       </c>
@@ -1745,12 +1745,12 @@
         <v>6</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B7" s="3"/>
       <c r="C7" s="3" t="s">
@@ -1760,29 +1760,29 @@
         <v>6</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
       <c r="E9" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
@@ -1797,18 +1797,18 @@
         <v>63</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="57" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="28.5" x14ac:dyDescent="0.2">
@@ -1823,12 +1823,12 @@
         <v>6</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3" t="s">
@@ -1838,27 +1838,27 @@
         <v>31</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>80</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="7" t="s">
@@ -1868,12 +1868,12 @@
         <v>33</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B16" s="8" t="s">
         <v>5</v>
@@ -1885,7 +1885,7 @@
         <v>6</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -1925,21 +1925,21 @@
     </row>
     <row r="2" spans="1:4" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="10" t="s">
         <v>127</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>5</v>
@@ -1953,7 +1953,7 @@
     </row>
     <row r="4" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>5</v>
@@ -1967,7 +1967,7 @@
     </row>
     <row r="5" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>5</v>
@@ -1981,7 +1981,7 @@
     </row>
     <row r="6" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>5</v>
@@ -1990,7 +1990,7 @@
         <v>6</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed the locator issue and added few tests
</commit_message>
<xml_diff>
--- a/src/main/resources/testData/TestData.xlsx
+++ b/src/main/resources/testData/TestData.xlsx
@@ -4,13 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2445" windowWidth="15465" windowHeight="3030" tabRatio="500" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="2445" windowWidth="15465" windowHeight="3030" tabRatio="500" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="LoginTest" sheetId="1" r:id="rId1"/>
     <sheet name="CreateAccountTest" sheetId="2" r:id="rId2"/>
     <sheet name="ForgotPasswordTest" sheetId="3" r:id="rId3"/>
     <sheet name="LogoutTest" sheetId="4" r:id="rId4"/>
+    <sheet name="DashboardTest" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0" iterateDelta="1E-4"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="136">
   <si>
     <t>Function</t>
   </si>
@@ -310,9 +311,6 @@
   </si>
   <si>
     <t>testEmptyPasswordField</t>
-  </si>
-  <si>
-    <t>testPasswordTooShort</t>
   </si>
   <si>
     <t>password
@@ -453,6 +451,23 @@
   </si>
   <si>
     <t>Email already registered.</t>
+  </si>
+  <si>
+    <t>bigbignoopavi@yopmail.com</t>
+  </si>
+  <si>
+    <t>testDashboardPage</t>
+  </si>
+  <si>
+    <t>testTaskHomeProfilePage</t>
+  </si>
+  <si>
+    <t>My Tasks
+john
+Sign in to your account</t>
+  </si>
+  <si>
+    <t>testVerfiySideButton</t>
   </si>
 </sst>
 </file>
@@ -867,7 +882,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>13</v>
       </c>
@@ -877,8 +892,8 @@
       <c r="C5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>96</v>
+      <c r="D5" s="4" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
@@ -906,7 +921,7 @@
         <v>6</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
@@ -916,17 +931,17 @@
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
@@ -936,7 +951,7 @@
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
@@ -946,7 +961,7 @@
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
@@ -956,7 +971,7 @@
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
@@ -984,7 +999,7 @@
         <v>27</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
@@ -1125,7 +1140,7 @@
     </row>
     <row r="25" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>5</v>
@@ -1139,7 +1154,7 @@
     </row>
     <row r="26" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>5</v>
@@ -1185,7 +1200,7 @@
         <v>47</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>1</v>
@@ -1266,7 +1281,7 @@
         <v>58</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
@@ -1289,7 +1304,7 @@
         <v>58</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
@@ -1358,12 +1373,12 @@
         <v>6</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="85.5" x14ac:dyDescent="0.2">
       <c r="A9" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -1371,7 +1386,7 @@
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
       <c r="G9" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
@@ -1384,7 +1399,7 @@
       <c r="C10" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="8" t="s">
         <v>70</v>
       </c>
       <c r="E10" s="3" t="s">
@@ -1417,7 +1432,7 @@
         <v>6</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
@@ -1445,30 +1460,30 @@
     </row>
     <row r="13" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>33</v>
       </c>
       <c r="C13" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="G13" s="3" t="s">
         <v>110</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>36</v>
@@ -1486,7 +1501,7 @@
         <v>36</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
@@ -1540,10 +1555,10 @@
         <v>82</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>5</v>
@@ -1581,9 +1596,9 @@
         <v>83</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" ht="85.5" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>49</v>
@@ -1594,15 +1609,15 @@
       <c r="D19" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="E19" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="F19" s="3"/>
+      <c r="G19" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="14.25" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="1:7" ht="85.5" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>69</v>
       </c>
@@ -1610,10 +1625,10 @@
         <v>67</v>
       </c>
       <c r="C20" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="D20" s="4" t="s">
         <v>119</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>120</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>6</v>
@@ -1636,7 +1651,7 @@
         <v>61</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>6</v>
@@ -1652,9 +1667,10 @@
   <hyperlinks>
     <hyperlink ref="D19" r:id="rId1"/>
     <hyperlink ref="D21" r:id="rId2" display="Avinash.Noop_Doddu@example.com"/>
+    <hyperlink ref="D10" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.74791666666666701" right="0.74791666666666701" top="0.98402777777777795" bottom="0.98402777777777795" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId4"/>
 </worksheet>
 </file>
 
@@ -1693,7 +1709,7 @@
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
@@ -1704,7 +1720,7 @@
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
@@ -1718,12 +1734,12 @@
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="71.25" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>70</v>
+      <c r="B5" s="4" t="s">
+        <v>119</v>
       </c>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
@@ -1733,11 +1749,11 @@
     </row>
     <row r="6" spans="1:5" ht="57" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>123</v>
-      </c>
       <c r="C6" s="3" t="s">
         <v>6</v>
       </c>
@@ -1745,7 +1761,7 @@
         <v>6</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
@@ -1760,7 +1776,7 @@
         <v>6</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
@@ -1771,7 +1787,7 @@
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
       <c r="E8" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
@@ -1779,10 +1795,14 @@
         <v>93</v>
       </c>
       <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
+      <c r="C9" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>6</v>
+      </c>
       <c r="E9" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
@@ -1797,7 +1817,7 @@
         <v>63</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="57" x14ac:dyDescent="0.2">
@@ -1808,7 +1828,7 @@
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
       <c r="E11" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="28.5" x14ac:dyDescent="0.2">
@@ -1823,7 +1843,7 @@
         <v>6</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
@@ -1841,19 +1861,19 @@
         <v>73</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" ht="199.5" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
-        <v>95</v>
+        <v>115</v>
       </c>
       <c r="B14" s="3"/>
-      <c r="C14" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>80</v>
+      <c r="C14" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
@@ -1873,10 +1893,10 @@
     </row>
     <row r="16" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A16" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>5</v>
+        <v>131</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>6</v>
@@ -1885,12 +1905,12 @@
         <v>6</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B5" r:id="rId1"/>
+    <hyperlink ref="B5" r:id="rId1" display="john.doe@exampl"/>
     <hyperlink ref="B16" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.74791666666666701" right="0.74791666666666701" top="0.98402777777777795" bottom="0.98402777777777795" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1925,21 +1945,21 @@
     </row>
     <row r="2" spans="1:4" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="10" t="s">
         <v>126</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B3" s="9" t="s">
         <v>5</v>
@@ -1953,7 +1973,7 @@
     </row>
     <row r="4" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>5</v>
@@ -1967,7 +1987,7 @@
     </row>
     <row r="5" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>5</v>
@@ -1981,7 +2001,7 @@
     </row>
     <row r="6" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>5</v>
@@ -1990,7 +2010,7 @@
         <v>6</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -2003,4 +2023,80 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="51" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B4" r:id="rId1"/>
+    <hyperlink ref="D4" r:id="rId2"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>